<commit_message>
operational csv for softwarex
</commit_message>
<xml_diff>
--- a/parameters/UA/ammonia/country_parameters.xlsx
+++ b/parameters/UA/ammonia/country_parameters.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\engs2859\Desktop\Geo-X\Geo-X\parameters\UA\ammonia\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unioxfordnexus-my.sharepoint.com/personal/engs2859_ox_ac_uk/Documents/Geo-X/Geo-X/parameters/UA/ammonia/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CD71765-3029-4097-9D5C-5CFDB476EAF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{88A4EBDB-4368-4A69-B424-380625435D0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D0CB3539-DEF2-BA4C-8A4E-4403EC5D0374}"/>
   <bookViews>
-    <workbookView xWindow="3510" yWindow="3510" windowWidth="21600" windowHeight="6150" xr2:uid="{60BD1E41-9A81-F547-A629-52DD9269BE2D}"/>
+    <workbookView xWindow="2740" yWindow="2740" windowWidth="18900" windowHeight="10960" xr2:uid="{60BD1E41-9A81-F547-A629-52DD9269BE2D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -435,24 +435,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A655327-FB0F-D040-A870-A9F18A82B881}">
   <dimension ref="A1:O2"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="8.125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="20.5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="16" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.83203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.1640625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="16" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="23.375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="25.875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="23.33203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="25.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -499,7 +499,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -510,31 +510,31 @@
         <v>0.02</v>
       </c>
       <c r="D2">
-        <v>0.161</v>
+        <v>0.11899999999999999</v>
       </c>
       <c r="E2">
         <v>20</v>
       </c>
       <c r="F2">
-        <v>0.161</v>
+        <v>0.11899999999999999</v>
       </c>
       <c r="G2">
         <v>20</v>
       </c>
       <c r="H2">
-        <v>0.161</v>
+        <v>0.11899999999999999</v>
       </c>
       <c r="I2">
         <v>20</v>
       </c>
       <c r="L2">
-        <v>0.161</v>
+        <v>0.11899999999999999</v>
       </c>
       <c r="M2">
         <v>20</v>
       </c>
       <c r="N2">
-        <v>0.161</v>
+        <v>0.11899999999999999</v>
       </c>
       <c r="O2">
         <v>50</v>

</xml_diff>